<commit_message>
more la prediction work - WTP nearly done
</commit_message>
<xml_diff>
--- a/pages/WR_progressions/Medals_Women_TP.xlsx
+++ b/pages/WR_progressions/Medals_Women_TP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\WR_progressions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9EE33E3-FF9D-47A4-B750-2CB8CE8D5E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCE0D1D1-D69C-4DDD-A218-EBB12CBE39AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{CC4DF8B1-FDE8-46DE-898D-C50D7CB0E2AF}"/>
+    <workbookView xWindow="25490" yWindow="15750" windowWidth="19420" windowHeight="10300" xr2:uid="{CC4DF8B1-FDE8-46DE-898D-C50D7CB0E2AF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>8th</t>
   </si>
@@ -78,6 +78,48 @@
   </si>
   <si>
     <t>Fastest_Seconds</t>
+  </si>
+  <si>
+    <t>DateSerial</t>
+  </si>
+  <si>
+    <t>Ballerup</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>Glasgow</t>
+  </si>
+  <si>
+    <t>Roubaix</t>
+  </si>
+  <si>
+    <t>Tokyo</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Pruszkow</t>
+  </si>
+  <si>
+    <t>Apeldoorn</t>
+  </si>
+  <si>
+    <t>Hong Kong</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>Rio de Janeiro</t>
+  </si>
+  <si>
+    <t>Cali</t>
+  </si>
+  <si>
+    <t>Location</t>
   </si>
 </sst>
 </file>
@@ -464,20 +506,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1400477D-CA59-426F-9BF4-08585135C868}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="9.1328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.73046875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.3984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.73046875" customWidth="1"/>
+    <col min="4" max="7" width="9.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.73046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -485,639 +529,729 @@
         <v>4</v>
       </c>
       <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2024</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="2">
         <v>2.915138888888889E-3</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>2.9120601851851851E-3</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>2.9220717592592592E-3</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>3.1005439814814815E-3</v>
       </c>
-      <c r="G2" s="3">
+      <c r="H2" s="3">
         <v>251.86799999999999</v>
       </c>
-      <c r="H2" s="3">
+      <c r="I2" s="3">
         <v>251.60199999999998</v>
       </c>
-      <c r="I2" s="3">
+      <c r="J2" s="3">
         <v>252.46699999999998</v>
       </c>
-      <c r="J2" s="3">
+      <c r="K2" s="3">
         <v>267.887</v>
       </c>
-      <c r="K2" s="2">
+      <c r="L2" s="2">
         <v>2.9120601851851851E-3</v>
       </c>
-      <c r="L2">
-        <f>K2*86400</f>
+      <c r="M2">
+        <f>L2*86400</f>
         <v>251.60199999999998</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N2">
+        <v>45581</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2024</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="2">
         <v>2.8319328703703705E-3</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3" s="2">
         <v>2.8384027777777778E-3</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>2.855439814814815E-3</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>2.9190393518518519E-3</v>
       </c>
-      <c r="G3" s="3">
-        <f>C3*86400</f>
+      <c r="H3" s="3">
+        <f>D3*86400</f>
         <v>244.679</v>
       </c>
-      <c r="H3" s="3">
-        <f t="shared" ref="H3:J3" si="0">D3*86400</f>
+      <c r="I3" s="3">
+        <f t="shared" ref="I3:K3" si="0">E3*86400</f>
         <v>245.238</v>
       </c>
-      <c r="I3" s="3">
+      <c r="J3" s="3">
         <f t="shared" si="0"/>
         <v>246.71</v>
       </c>
-      <c r="J3" s="3">
+      <c r="K3" s="3">
         <f t="shared" si="0"/>
         <v>252.20500000000001</v>
       </c>
-      <c r="K3" s="2">
+      <c r="L3" s="2">
         <v>2.8276157407407408E-3</v>
       </c>
-      <c r="L3">
-        <f t="shared" ref="L3:L15" si="1">K3*86400</f>
+      <c r="M3">
+        <f t="shared" ref="M3:M15" si="1">L3*86400</f>
         <v>244.30600000000001</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N3">
+        <v>45511</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2023</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2">
         <v>2.8973726851851851E-3</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4" s="2">
         <v>2.9140856481481479E-3</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="2">
         <v>2.9419444444444445E-3</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4" s="2">
         <v>3.0000925925925924E-3</v>
       </c>
-      <c r="G4">
-        <f>C4*86400</f>
+      <c r="H4">
+        <f>D4*86400</f>
         <v>250.333</v>
       </c>
-      <c r="H4">
-        <f t="shared" ref="H4:J15" si="2">D4*86400</f>
+      <c r="I4">
+        <f t="shared" ref="I4:K15" si="2">E4*86400</f>
         <v>251.77699999999999</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f t="shared" si="2"/>
         <v>254.184</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <f t="shared" si="2"/>
         <v>259.20799999999997</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>2.8792939814814818E-3</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <f t="shared" si="1"/>
         <v>248.77100000000002</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N4">
+        <v>45141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2022</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="2">
         <v>2.9052199074074071E-3</v>
       </c>
-      <c r="D5" s="2">
+      <c r="E5" s="2">
         <v>2.9295949074074072E-3</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="2">
         <v>2.9331597222222224E-3</v>
       </c>
-      <c r="F5" s="2">
+      <c r="G5" s="2">
         <v>2.9990625000000004E-3</v>
       </c>
-      <c r="G5">
-        <f t="shared" ref="G5:G15" si="3">C5*86400</f>
+      <c r="H5">
+        <f t="shared" ref="H5:H15" si="3">D5*86400</f>
         <v>251.01099999999997</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f t="shared" si="2"/>
         <v>253.11699999999999</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f t="shared" si="2"/>
         <v>253.42500000000001</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <f t="shared" si="2"/>
         <v>259.11900000000003</v>
       </c>
-      <c r="K5" s="2">
+      <c r="L5" s="2">
         <v>2.8907407407407406E-3</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <f t="shared" si="1"/>
         <v>249.76</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N5">
+        <v>44847</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2021</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2">
         <v>2.9291898148148146E-3</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6" s="2">
         <v>2.9418518518518517E-3</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="2">
         <v>2.9652777777777776E-3</v>
       </c>
-      <c r="F6" s="2">
+      <c r="G6" s="2">
         <v>3.1755787037037039E-3</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f t="shared" si="3"/>
         <v>253.08199999999999</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f t="shared" si="2"/>
         <v>254.17599999999999</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f t="shared" si="2"/>
         <v>256.2</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <f t="shared" si="2"/>
         <v>274.37</v>
       </c>
-      <c r="K6" s="2">
+      <c r="L6" s="2">
         <v>2.8790740740740743E-3</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <f t="shared" si="1"/>
         <v>248.75200000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N6">
+        <v>44490</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2021</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2">
         <v>2.8623495370370369E-3</v>
       </c>
-      <c r="D7" s="2">
+      <c r="E7" s="2">
         <v>2.8821990740740739E-3</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="2">
         <v>2.8948842592592594E-3</v>
       </c>
-      <c r="F7" s="2">
+      <c r="G7" s="2">
         <v>2.9610185185185186E-3</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <f t="shared" si="3"/>
         <v>247.30699999999999</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f t="shared" si="2"/>
         <v>249.02199999999999</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f t="shared" si="2"/>
         <v>250.11800000000002</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <f t="shared" si="2"/>
         <v>255.83200000000002</v>
       </c>
-      <c r="K7" s="2">
+      <c r="L7" s="2">
         <v>2.826875E-3</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <f t="shared" si="1"/>
         <v>244.24199999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N7">
+        <v>44412</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2020</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2">
         <v>2.9077430555555553E-3</v>
       </c>
-      <c r="D8" s="2">
+      <c r="E8" s="2">
         <v>2.915173611111111E-3</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="2">
         <v>2.9250925925925928E-3</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <v>3.0250925925925927E-3</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <f t="shared" si="3"/>
         <v>251.22899999999998</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f t="shared" si="2"/>
         <v>251.87099999999998</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f t="shared" si="2"/>
         <v>252.72800000000001</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <f t="shared" si="2"/>
         <v>261.36799999999999</v>
       </c>
-      <c r="K8" s="2">
+      <c r="L8" s="2">
         <v>2.9055439814814812E-3</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <f t="shared" si="1"/>
         <v>251.03899999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N8">
+        <v>43889</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2019</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="2">
         <v>2.9504050925925926E-3</v>
       </c>
-      <c r="D9" s="2">
+      <c r="E9" s="2">
         <v>2.9585416666666666E-3</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="2">
         <v>2.9984374999999998E-3</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9" s="2">
         <v>3.0766782407407405E-3</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <f t="shared" si="3"/>
         <v>254.91499999999999</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <f t="shared" si="2"/>
         <v>255.61799999999999</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <f t="shared" si="2"/>
         <v>259.065</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <f t="shared" si="2"/>
         <v>265.82499999999999</v>
       </c>
-      <c r="K9" s="2">
+      <c r="L9" s="2">
         <v>2.9436689814814816E-3</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <f t="shared" si="1"/>
         <v>254.333</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N9">
+        <v>43524</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2018</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2">
         <v>2.9957870370370373E-3</v>
       </c>
-      <c r="D10" s="2">
+      <c r="E10" s="2">
         <v>2.9997337962962963E-3</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="2">
         <v>3.0271180555555555E-3</v>
       </c>
-      <c r="F10" s="2">
+      <c r="G10" s="2">
         <v>3.1226736111111108E-3</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <f t="shared" si="3"/>
         <v>258.83600000000001</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <f t="shared" si="2"/>
         <v>259.17700000000002</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <f t="shared" si="2"/>
         <v>261.54300000000001</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <f t="shared" si="2"/>
         <v>269.79899999999998</v>
       </c>
-      <c r="K10" s="2">
+      <c r="L10" s="2">
         <v>2.9591319444444448E-3</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <f t="shared" si="1"/>
         <v>255.66900000000004</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N10">
+        <v>43159</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2017</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2">
         <v>2.9828935185185184E-3</v>
       </c>
-      <c r="D11" s="2">
+      <c r="E11" s="2">
         <v>2.9937384259259257E-3</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11" s="2">
         <v>3.003645833333333E-3</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G11" s="2">
         <v>3.1079050925925927E-3</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <f t="shared" si="3"/>
         <v>257.72199999999998</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <f t="shared" si="2"/>
         <v>258.65899999999999</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <f t="shared" si="2"/>
         <v>259.51499999999999</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <f t="shared" si="2"/>
         <v>268.52300000000002</v>
       </c>
-      <c r="K11" s="2">
+      <c r="L11" s="2">
         <v>2.9828935185185184E-3</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <f t="shared" si="1"/>
         <v>257.72199999999998</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N11">
+        <v>42837</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2016</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="2">
         <v>2.9650462962962964E-3</v>
       </c>
-      <c r="D12" s="2">
+      <c r="E12" s="2">
         <v>3.0169444444444445E-3</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12" s="2">
         <v>3.017048611111111E-3</v>
       </c>
-      <c r="F12" s="2">
+      <c r="G12" s="2">
         <v>3.1243171296296292E-3</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <f t="shared" si="3"/>
         <v>256.18</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <f t="shared" si="2"/>
         <v>260.66399999999999</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <f t="shared" si="2"/>
         <v>260.673</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <f t="shared" si="2"/>
         <v>269.94099999999997</v>
       </c>
-      <c r="K12" s="2">
+      <c r="L12" s="2">
         <v>2.9491435185185185E-3</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <f t="shared" si="1"/>
         <v>254.80599999999998</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N12">
+        <v>42435</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>2016</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="2">
         <v>2.9312499999999998E-3</v>
       </c>
-      <c r="D13" s="2">
+      <c r="E13" s="2">
         <v>2.943125E-3</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="2">
         <v>2.9983680555555558E-3</v>
       </c>
-      <c r="F13" s="2">
+      <c r="G13" s="2">
         <v>3.1132870370370372E-3</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <f t="shared" si="3"/>
         <v>253.26</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <f t="shared" si="2"/>
         <v>254.286</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <f t="shared" si="2"/>
         <v>259.05900000000003</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <f t="shared" si="2"/>
         <v>268.988</v>
       </c>
-      <c r="K13" s="2">
+      <c r="L13" s="2">
         <v>2.89625E-3</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <f t="shared" si="1"/>
         <v>250.23599999999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N13">
+        <v>42593</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2015</v>
       </c>
       <c r="B14" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D14" s="2">
         <v>2.9876736111111111E-3</v>
       </c>
-      <c r="D14" s="2">
+      <c r="E14" s="2">
         <v>2.9885069444444442E-3</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14" s="2">
         <v>3.0173495370370371E-3</v>
       </c>
-      <c r="F14" s="2">
+      <c r="G14" s="2">
         <v>3.1504398148148147E-3</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <f t="shared" si="3"/>
         <v>258.13499999999999</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <f t="shared" si="2"/>
         <v>258.20699999999999</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <f t="shared" si="2"/>
         <v>260.69900000000001</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <f t="shared" si="2"/>
         <v>272.19799999999998</v>
       </c>
-      <c r="K14" s="2">
+      <c r="L14" s="2">
         <v>2.9361458333333331E-3</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <f t="shared" si="1"/>
         <v>253.68299999999999</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="N14">
+        <v>42053</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2014</v>
       </c>
       <c r="B15" t="s">
         <v>6</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="2">
         <v>3.1087615740740737E-3</v>
       </c>
-      <c r="D15" s="2">
+      <c r="E15" s="2">
         <v>3.1333449074074076E-3</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="2">
         <v>3.1424074074074076E-3</v>
       </c>
-      <c r="F15" s="2">
+      <c r="G15" s="2">
         <v>3.2786921296296297E-3</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <f t="shared" si="3"/>
         <v>268.59699999999998</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <f t="shared" si="2"/>
         <v>270.721</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <f t="shared" si="2"/>
         <v>271.50400000000002</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <f t="shared" si="2"/>
         <v>283.279</v>
       </c>
-      <c r="K15" s="2">
+      <c r="L15" s="2">
         <v>3.0486921296296295E-3</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <f t="shared" si="1"/>
         <v>263.40699999999998</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="C16" s="1"/>
+      <c r="N15">
+        <v>41696</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>